<commit_message>
docs: Punto 4 y Corrección Punto 1
</commit_message>
<xml_diff>
--- a/docs/Asignación el Equipo de Producto - Definición del contrato de la API.xlsx
+++ b/docs/Asignación el Equipo de Producto - Definición del contrato de la API.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebastian.granados-l\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebastian.granados-l\Documents\DOSW_ParcialT2_SebastianGranados\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FECBD41E-9E47-4A70-887B-805C683F03B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F99D8F6-6F3F-48BE-A188-62F0D454D80C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{7519990D-B813-46C2-8091-3D5E6CABC3BD}"/>
   </bookViews>
@@ -125,15 +125,9 @@
     <t>Si</t>
   </si>
   <si>
-    <t>{Barbero: "Miguel", fecha: "10-11-2026", hora: "13:00"}</t>
-  </si>
-  <si>
     <t>String / Obligatoria</t>
   </si>
   <si>
-    <t>{Estado: "Disponible"}</t>
-  </si>
-  <si>
     <t>GET api/v1/turnos/{id}</t>
   </si>
   <si>
@@ -146,9 +140,6 @@
     <t>String / Obligatorio</t>
   </si>
   <si>
-    <t>String, fechaHora/ Obligatorio</t>
-  </si>
-  <si>
     <t>{idTurno: "01"}</t>
   </si>
   <si>
@@ -161,9 +152,6 @@
     <t>String, FechaHora / Obligatoria</t>
   </si>
   <si>
-    <t>{idReserva: "01", fecha: "11-11-2026", hora: "15:00"}</t>
-  </si>
-  <si>
     <t>{idReserva: "01", Reserva: "CONFIRMADA"/"DENEGADA", Turno: "OCUPADO", Barbero: "Miguel"}</t>
   </si>
   <si>
@@ -176,7 +164,19 @@
     <t>{admin@gmail.com}</t>
   </si>
   <si>
-    <t>{Token: "AdgRftH32Jk89YT7"}</t>
+    <t>{idTurno: "01", Estado: "Disponible"}</t>
+  </si>
+  <si>
+    <t>String, Enum, fechaHora/ Obligatorio</t>
+  </si>
+  <si>
+    <t>{Barbero: "Miguel", Especialidades: "CORTE, CORTE CON BARBA", fecha: "Lunes a Jueves", hora: "10:00 a 17:00"}</t>
+  </si>
+  <si>
+    <t>{idReserva: "01", fecha: "11-11-2026", hora: "15:00", idReserva: "02", fecha: "15-12-2026", hora: "16:00"}</t>
+  </si>
+  <si>
+    <t>{Token: "AdgRftH32Jk89YT7", idLogin: "01"}</t>
   </si>
 </sst>
 </file>
@@ -258,7 +258,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -266,10 +266,20 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -595,7 +605,7 @@
     <col min="5" max="5" width="22" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="21" style="1" customWidth="1"/>
-    <col min="8" max="8" width="17.140625" style="1" customWidth="1"/>
+    <col min="8" max="8" width="19.42578125" style="1" customWidth="1"/>
     <col min="9" max="9" width="30.28515625" style="1" customWidth="1"/>
     <col min="10" max="10" width="20.85546875" style="1" customWidth="1"/>
   </cols>
@@ -629,146 +639,146 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B3" s="2" t="s">
+    <row r="3" spans="2:10" ht="120" x14ac:dyDescent="0.25">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="E3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="F3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="G3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" ht="114.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" s="5" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="90" x14ac:dyDescent="0.25">
+      <c r="B5" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I5" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J5" s="5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="120" x14ac:dyDescent="0.25">
+      <c r="B6" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="5"/>
+      <c r="F6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G6" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="H6" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="I6" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J6" s="5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="B7" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="I7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="I3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B4" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B6" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="2"/>
-      <c r="F6" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="J7" s="2" t="s">
+      <c r="J7" s="5" t="s">
         <v>42</v>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: Corrección punto 1
</commit_message>
<xml_diff>
--- a/docs/Asignación el Equipo de Producto - Definición del contrato de la API.xlsx
+++ b/docs/Asignación el Equipo de Producto - Definición del contrato de la API.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebastian.granados-l\Documents\DOSW_ParcialT2_SebastianGranados\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F99D8F6-6F3F-48BE-A188-62F0D454D80C}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B03C38-4A15-49CF-9176-0DE802C4B3DD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{7519990D-B813-46C2-8091-3D5E6CABC3BD}"/>
   </bookViews>
@@ -152,15 +152,9 @@
     <t>String, FechaHora / Obligatoria</t>
   </si>
   <si>
-    <t>{idReserva: "01", Reserva: "CONFIRMADA"/"DENEGADA", Turno: "OCUPADO", Barbero: "Miguel"}</t>
-  </si>
-  <si>
     <t>{Cliente: "Juan Perez", idReserva: "01", fecha: "11-11-2026", hora: "15:00", Cliente: "Ernesto Vergara", idReserva: "02", fecha: "11-11-2026", hora: "15:00"}</t>
   </si>
   <si>
-    <t>{idReserva: "01", idReserva: "02"}</t>
-  </si>
-  <si>
     <t>{admin@gmail.com}</t>
   </si>
   <si>
@@ -173,10 +167,16 @@
     <t>{Barbero: "Miguel", Especialidades: "CORTE, CORTE CON BARBA", fecha: "Lunes a Jueves", hora: "10:00 a 17:00"}</t>
   </si>
   <si>
-    <t>{idReserva: "01", fecha: "11-11-2026", hora: "15:00", idReserva: "02", fecha: "15-12-2026", hora: "16:00"}</t>
-  </si>
-  <si>
     <t>{Token: "AdgRftH32Jk89YT7", idLogin: "01"}</t>
+  </si>
+  <si>
+    <t>{idReserva: "SER-001", Reserva: "CONFIRMADA"/"DENEGADA", Turno: "OCUPADO", Barbero: "Miguel"}</t>
+  </si>
+  <si>
+    <t>{idReserva: "SER-003", fecha: "11-11-2026", hora: "15:00", idReserva: "SER-005", fecha: "15-12-2026", hora: "16:00"}</t>
+  </si>
+  <si>
+    <t>{idReserva: "SER-003", idReserva: "SER-005"}</t>
   </si>
 </sst>
 </file>
@@ -605,7 +605,7 @@
     <col min="5" max="5" width="22" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="21" style="1" customWidth="1"/>
-    <col min="8" max="8" width="19.42578125" style="1" customWidth="1"/>
+    <col min="8" max="8" width="23.85546875" style="1" customWidth="1"/>
     <col min="9" max="9" width="30.28515625" style="1" customWidth="1"/>
     <col min="10" max="10" width="20.85546875" style="1" customWidth="1"/>
   </cols>
@@ -639,7 +639,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="120" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:10" ht="105" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
@@ -656,16 +656,16 @@
         <v>13</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="I3" s="5" t="s">
         <v>25</v>
       </c>
       <c r="J3" s="5" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4" spans="2:10" ht="114.75" x14ac:dyDescent="0.25">
@@ -694,7 +694,7 @@
         <v>25</v>
       </c>
       <c r="J4" s="5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="2:10" ht="90" x14ac:dyDescent="0.25">
@@ -744,13 +744,13 @@
         <v>31</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="I6" s="5" t="s">
         <v>33</v>
       </c>
       <c r="J6" s="5" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="76.5" x14ac:dyDescent="0.25">
@@ -773,13 +773,13 @@
         <v>29</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I7" s="5" t="s">
         <v>25</v>
       </c>
       <c r="J7" s="5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Parcial T2 - Corrección puntos 1 y 4
</commit_message>
<xml_diff>
--- a/docs/Asignación el Equipo de Producto - Definición del contrato de la API.xlsx
+++ b/docs/Asignación el Equipo de Producto - Definición del contrato de la API.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sebastian.granados-l\Documents\DOSW_ParcialT2_SebastianGranados\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kamil\Desktop\Escritorio\DOSW\DOSW_ParcialT2_SebastianGranados\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32B03C38-4A15-49CF-9176-0DE802C4B3DD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1C2CC60-0DDE-42ED-A688-39719A9FB711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="12105" xr2:uid="{7519990D-B813-46C2-8091-3D5E6CABC3BD}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{7519990D-B813-46C2-8091-3D5E6CABC3BD}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="45">
   <si>
     <t>Método y Ruta</t>
   </si>
@@ -66,13 +66,43 @@
     <t>ADMIN</t>
   </si>
   <si>
-    <t>El barbero debe existir. La fecha debe ser futura y caer en un día de disponibilidad del barbero; la hora debe estar dentro de su horario. No se duplica barbero + fecha + hora.</t>
-  </si>
-  <si>
-    <t>El turno nace DISPONIBLE.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Si todas pasan: la reserva queda CONFIRMADA, el turno OCUPADO y el total es la suma de los servicios. </t>
+    <t>Consulta las reservas de todos los clientes, pasadas y futuras, ordenadas por fecha y hora de manera descendente. </t>
+  </si>
+  <si>
+    <t>Los usuarios administrador y los clientes son usuarios predefinidos que tienen que crear por medio de Base de datos, con su correo y contraseña.</t>
+  </si>
+  <si>
+    <t>POST api/v1/reservas</t>
+  </si>
+  <si>
+    <t>CLIENTE</t>
+  </si>
+  <si>
+    <t>Si</t>
+  </si>
+  <si>
+    <t>CLIENTE, ADMIN</t>
+  </si>
+  <si>
+    <t>String, FechaHora / Obligatoria</t>
+  </si>
+  <si>
+    <t>El barbero debe existir.La fecha debe ser futura y caer en un día de disponibilidad del barbero; la hora debe estar dentro de su horario. No se duplica barbero + fecha + hora. El turno se Crea en Estado Disponible</t>
+  </si>
+  <si>
+    <t>barberoId no vacio. fecha Obligatoria y hora Obligatoria</t>
+  </si>
+  <si>
+    <t>{barberoId: "01", Especialidades: "CORTE, CORTE CON BARBA", fecha: "Lunes a Jueves", hora: "10:00 a 17:00"}</t>
+  </si>
+  <si>
+    <t>Id, barbero, fecha y hora</t>
+  </si>
+  <si>
+    <t>barberoId, Especialidades, Fecha y Hora-Todos Obligatorios</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fecha y hora obligatorios así como servicios no vacío. </t>
   </si>
   <si>
     <r>
@@ -97,93 +127,69 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (sección 4). Si hay alguna falla, el proceso se detiene y retorna el motivo específico. Sin preferencia de barbero, el sistema asigna uno disponible con la especialidad requerida.</t>
+      <t xml:space="preserve"> (sección 4). Si hay alguna falla, el proceso se detiene y retorna el motivo específico. Incluye: Franja con menos de 3 reservas y un turno disponible, datos del cliente, barbero libre con la especialidad requerida.</t>
     </r>
   </si>
   <si>
-    <t>Consulta únicamente las reservas del cliente autenticado; su identidad se obtiene de la sesión token, no de un identificador enviado por el cliente.</t>
-  </si>
-  <si>
-    <t>Incluye todas las reservas realizadas por ese usuario, ordenadas por fecha y hora de manera descendente.</t>
-  </si>
-  <si>
-    <t>Consulta las reservas de todos los clientes, pasadas y futuras, ordenadas por fecha y hora de manera descendente. </t>
-  </si>
-  <si>
-    <t>El usuario puede iniciar sesión para acceder a las funcionalidades que tiene permitidas.</t>
-  </si>
-  <si>
-    <t>Los usuarios administrador y los clientes son usuarios predefinidos que tienen que crear por medio de Base de datos, con su correo y contraseña.</t>
-  </si>
-  <si>
-    <t>POST api/v1/reservas</t>
-  </si>
-  <si>
-    <t>CLIENTE</t>
-  </si>
-  <si>
-    <t>Si</t>
-  </si>
-  <si>
-    <t>String / Obligatoria</t>
-  </si>
-  <si>
-    <t>GET api/v1/turnos/{id}</t>
-  </si>
-  <si>
-    <t>GET api/v1/turnos/**</t>
-  </si>
-  <si>
-    <t>CLIENTE, ADMIN</t>
-  </si>
-  <si>
-    <t>String / Obligatorio</t>
-  </si>
-  <si>
-    <t>{idTurno: "01"}</t>
-  </si>
-  <si>
-    <t>String / Opcional</t>
-  </si>
-  <si>
-    <t>{idTurno: "02"}</t>
-  </si>
-  <si>
-    <t>String, FechaHora / Obligatoria</t>
-  </si>
-  <si>
-    <t>{Cliente: "Juan Perez", idReserva: "01", fecha: "11-11-2026", hora: "15:00", Cliente: "Ernesto Vergara", idReserva: "02", fecha: "11-11-2026", hora: "15:00"}</t>
-  </si>
-  <si>
-    <t>{admin@gmail.com}</t>
-  </si>
-  <si>
-    <t>{idTurno: "01", Estado: "Disponible"}</t>
-  </si>
-  <si>
-    <t>String, Enum, fechaHora/ Obligatorio</t>
-  </si>
-  <si>
-    <t>{Barbero: "Miguel", Especialidades: "CORTE, CORTE CON BARBA", fecha: "Lunes a Jueves", hora: "10:00 a 17:00"}</t>
-  </si>
-  <si>
-    <t>{Token: "AdgRftH32Jk89YT7", idLogin: "01"}</t>
-  </si>
-  <si>
-    <t>{idReserva: "SER-001", Reserva: "CONFIRMADA"/"DENEGADA", Turno: "OCUPADO", Barbero: "Miguel"}</t>
-  </si>
-  <si>
-    <t>{idReserva: "SER-003", fecha: "11-11-2026", hora: "15:00", idReserva: "SER-005", fecha: "15-12-2026", hora: "16:00"}</t>
-  </si>
-  <si>
-    <t>{idReserva: "SER-003", idReserva: "SER-005"}</t>
+    <t>fecha, hora, servicios, barberoId, nombre, telefono y correo.</t>
+  </si>
+  <si>
+    <t>{fecha:"2026-11-12",hora:"11:00",servicios:["SER-001","SER-004"],nombre:"Juan Pérez",telefono:"3001234567",correo:"juan.perez@gmail.com"}</t>
+  </si>
+  <si>
+    <t>{idTurno: "TUR-001", barbero: "Miguel", fecha: "11-12-2026", hora: "15:00", Estado: "DISPONIBLE"}</t>
+  </si>
+  <si>
+    <t>Id, estado, turnoId, barbero, fecha, hora, servicios y total / Todos Obligatorios</t>
+  </si>
+  <si>
+    <t>{idReserva: "RES-001", estado: "CONFIRMADA"/"DENEGADA", Turno: "OCUPADO", barbero:"Andrés",fecha:"2026-11-12",hora:"11:00",servicios:["SER-001","SER-004"],total:45000}</t>
+  </si>
+  <si>
+    <t>Se identifica con el token y solo se devuelven sus reservas.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GET api/v1/reservas </t>
+  </si>
+  <si>
+    <t>{idReserva: "RES-003", fecha: "11-11-2026", hora: "15:00"} {idReserva: "SER-005", fecha: "15-12-2026", hora: "16:00"}</t>
+  </si>
+  <si>
+    <t>Id, Fecha y Hora / Son Obligatorias</t>
+  </si>
+  <si>
+    <t>GET api/v1/reservas/me</t>
+  </si>
+  <si>
+    <t>Un token válido</t>
+  </si>
+  <si>
+    <t>GET api/v1/reservas</t>
+  </si>
+  <si>
+    <t>{Cliente: "Juan Perez", idReserva: "RES-001", fecha: "11-11-2026", hora: "15:00", Cliente: "Ernesto Vergara", idReserva: "RES-002", fecha: "11-11-2026", hora: "15:00"}</t>
+  </si>
+  <si>
+    <t>El usuario puede iniciar sesión para acceder a las funcionalidades que tiene permitidas. La contraseña y el correo son obligatorios</t>
+  </si>
+  <si>
+    <t>correo y password / Son obligatorio</t>
+  </si>
+  <si>
+    <t>{correo:"admin@gmail.com",password:"Admin123*"}</t>
+  </si>
+  <si>
+    <t>token, tipo, rol/ Obligatoria</t>
+  </si>
+  <si>
+    <t>{Token: "AdgRftH32Jk89YT7", tipo:"Bearer", rol: "ADMIN", idLogin: "LOG-001"}</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -217,6 +223,12 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -266,9 +278,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -281,9 +290,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -300,9 +312,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -340,7 +352,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -446,7 +458,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -588,7 +600,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -597,7 +609,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09F3E740-5ECB-4195-A099-841B3BEFCBFA}">
   <dimension ref="B2:J7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34" style="1" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" style="1" customWidth="1"/>
@@ -605,9 +617,9 @@
     <col min="5" max="5" width="22" style="1" customWidth="1"/>
     <col min="6" max="6" width="23.7109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="21" style="1" customWidth="1"/>
-    <col min="8" max="8" width="23.85546875" style="1" customWidth="1"/>
+    <col min="8" max="8" width="35.5703125" style="1" customWidth="1"/>
     <col min="9" max="9" width="30.28515625" style="1" customWidth="1"/>
-    <col min="10" max="10" width="20.85546875" style="1" customWidth="1"/>
+    <col min="10" max="10" width="27.140625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
@@ -639,152 +651,150 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" spans="2:10" ht="105" x14ac:dyDescent="0.25">
-      <c r="B3" s="3" t="s">
+    <row r="3" spans="2:10" ht="102" x14ac:dyDescent="0.25">
+      <c r="B3" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="D3" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="4" t="s">
+      <c r="E3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="I3" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="2:10" ht="135" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" ht="75" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="I5" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" ht="105" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="F6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="G3" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="H3" s="5" t="s">
+      <c r="G6" s="4"/>
+      <c r="H6" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="I3" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J3" s="5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="4" spans="2:10" ht="114.75" x14ac:dyDescent="0.25">
-      <c r="B4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J4" s="5" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="2:10" ht="90" x14ac:dyDescent="0.25">
-      <c r="B5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H5" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J5" s="5" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="6" spans="2:10" ht="120" x14ac:dyDescent="0.25">
-      <c r="B6" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" s="5"/>
-      <c r="F6" s="4" t="s">
+      <c r="I6" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G6" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>34</v>
+      <c r="J6" s="4" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="2:10" ht="76.5" x14ac:dyDescent="0.25">
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D7" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="I7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="J7" s="5" t="s">
-        <v>39</v>
+      <c r="D7" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="I7" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H7" r:id="rId1" xr:uid="{9B4211D2-FD34-4C23-8691-AD66B93DE1FF}"/>
+    <hyperlink ref="H7" r:id="rId1" display="{admin@gmail.com}" xr:uid="{9B4211D2-FD34-4C23-8691-AD66B93DE1FF}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId2"/>

</xml_diff>